<commit_message>
Auto update Pengadaan 2026-10-15 09:10:20
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-15).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-15).xlsx
@@ -1020,35 +1020,27 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E17" s="4" t="n">
+        <v>1</v>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>1796500000</v>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1170,35 +1162,27 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E20" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G20" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>3839600910</v>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
@@ -1324,13 +1308,13 @@
         <v>80</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>847942644</v>
+        <v>850708644</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>59461794</v>
+        <v>62227794</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>5</v>
@@ -1389,22 +1373,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>103</v>
+        <v>128</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>677290237</v>
+        <v>674360508</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>137583844</v>
+        <v>134654115</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>116218702</v>
+        <v>1345382085</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1423,22 +1407,22 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>507942073</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>338217900</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>338050900</v>
+        <v>3037348900</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>22</v>
@@ -1460,13 +1444,13 @@
         <v>130</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>993618445</v>
+        <v>990746345</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>41</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>351115088</v>
+        <v>348242988</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>41</v>
@@ -1528,13 +1512,13 @@
         <v>171</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2269571073</v>
+        <v>2260066920</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1136240668</v>
+        <v>1126736515</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1559,22 +1543,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>79101092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>75945607</v>
+        <v>225945607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>49</v>
@@ -1596,13 +1580,13 @@
         <v>55</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>335612543</v>
+        <v>335468518</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>30262050</v>
+        <v>30118025</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>5</v>
@@ -1630,13 +1614,13 @@
         <v>122</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>767894130</v>
+        <v>764274671</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>107342366</v>
+        <v>103722907</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1664,13 +1648,13 @@
         <v>42</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>292846882</v>
+        <v>204513748</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>108974684</v>
+        <v>20641550</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>5</v>
@@ -1732,13 +1716,13 @@
         <v>66</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>463972148</v>
+        <v>463836830</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>93366423</v>
+        <v>93231105</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>6</v>
@@ -1797,22 +1781,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>100</v>
+        <v>111</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>1227952291</v>
+        <v>847360391</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>461686502</v>
+        <v>81094602</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>451166160</v>
+        <v>1801299990</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>84</v>
@@ -1834,13 +1818,13 @@
         <v>97</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>384332451</v>
+        <v>382731831</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>11</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>87341338</v>
+        <v>85740718</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>11</v>
@@ -1868,13 +1852,13 @@
         <v>107</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1270987621</v>
+        <v>1245457621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>378058156</v>
+        <v>352528156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -1936,13 +1920,13 @@
         <v>82</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>737837746</v>
+        <v>724469682</v>
       </c>
       <c r="E41" s="4" t="n">
         <v>16</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>73061846</v>
+        <v>59693782</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>16</v>
@@ -2004,13 +1988,13 @@
         <v>50</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>708077545</v>
+        <v>727698127</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>34949904</v>
+        <v>54570486</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2035,22 +2019,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>151137140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>72726534</v>
+        <v>83626512</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>15</v>
@@ -2119,22 +2103,22 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1126161761</v>
+        <v>1174814171</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>124972901</v>
+        <v>173625311</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>121983128</v>
+        <v>318350703</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>169</v>
@@ -2240,13 +2224,13 @@
         <v>105</v>
       </c>
       <c r="D49" s="11" t="n">
-        <v>620146476</v>
+        <v>618221476</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>15</v>
       </c>
       <c r="F49" s="11" t="n">
-        <v>204940123</v>
+        <v>203015123</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>15</v>
@@ -2355,30 +2339,24 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -2904,13 +2882,13 @@
         <v>32</v>
       </c>
       <c r="D65" s="11" t="n">
-        <v>197795800</v>
+        <v>199016800</v>
       </c>
       <c r="E65" s="4" t="n">
         <v>8</v>
       </c>
       <c r="F65" s="11" t="n">
-        <v>45935987</v>
+        <v>47156987</v>
       </c>
       <c r="G65" s="4" t="n">
         <v>8</v>
@@ -3148,13 +3126,13 @@
         <v>20</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>181625201</v>
+        <v>174734876</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>35716900</v>
+        <v>28826575</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>2</v>
@@ -3179,22 +3157,22 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D72" s="9" t="n">
         <v>637283463</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>108000000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>158730000</v>
+        <v>2359971000</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>29</v>
@@ -3300,7 +3278,7 @@
         <v>92</v>
       </c>
       <c r="D75" s="11" t="n">
-        <v>1089002496</v>
+        <v>1054602496</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>18</v>
@@ -3318,7 +3296,7 @@
         <v>74</v>
       </c>
       <c r="J75" s="11" t="n">
-        <v>669128310</v>
+        <v>634728310</v>
       </c>
     </row>
     <row r="76" ht="45" customHeight="1">
@@ -3334,13 +3312,13 @@
         <v>151</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1482468770</v>
+        <v>1480218770</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>26</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>216235114</v>
+        <v>213985114</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>26</v>
@@ -3363,28 +3341,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3904</v>
+        <v>3955</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32785458887</v>
+        <v>32283625052</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>426</v>
+        <v>477</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6796598056</v>
+        <v>6329164221</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>426</v>
+        <v>477</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>6373363220.6</v>
+        <v>19914588683.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3478</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>25988860831</v>
+        <v>25954460831</v>
       </c>
     </row>
   </sheetData>
@@ -3805,13 +3783,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>428765330</v>
+        <v>413165330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>276710330</v>
+        <v>261110330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4245,45 +4223,29 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>199078500</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -4315,29 +4277,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>112000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>111200910</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>111200910</v>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -4606,28 +4584,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1566751699</v>
+        <v>1346095756</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1225542538</v>
+        <v>1004886595</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>896262562</v>
+        <v>852531955</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>896262562</v>
+        <v>852531955</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4852,28 +4830,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>538286000</v>
+        <v>388286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>288750000</v>
+        <v>138750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>288306000</v>
+        <v>138306000</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
@@ -5105,13 +5083,13 @@
         <v>13</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>1694840343</v>
+        <v>1667542131</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>913021368</v>
+        <v>885723156</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>7</v>
@@ -5202,34 +5180,34 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>3541045550</v>
+        <v>2613177050</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>2025090451</v>
+        <v>1097221951</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1975819523</v>
+        <v>1062482323</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>1581713573</v>
+        <v>852976373</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="L37" s="11" t="n">
-        <v>535415363</v>
+        <v>188207363</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>16</v>
@@ -5313,13 +5291,13 @@
         <v>37</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>4288626639</v>
+        <v>4277601639</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>24</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>2769384586</v>
+        <v>2758359586</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>24</v>
@@ -5584,28 +5562,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>595373450</v>
+        <v>523391100</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>417917650</v>
+        <v>345935300</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>198768000</v>
+        <v>187868022</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -5704,28 +5682,28 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>932380105</v>
+        <v>716222170</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>471330601</v>
+        <v>255172666</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>448555830</v>
+        <v>252188255</v>
       </c>
       <c r="I46" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J46" s="9" t="n">
-        <v>309615830</v>
+        <v>113248255</v>
       </c>
       <c r="K46" s="10" t="inlineStr">
         <is>
@@ -6048,28 +6026,40 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>660566066</v>
-      </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="F52" s="9" t="n">
-        <v>340582172</v>
-      </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
-      </c>
-      <c r="I52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="J52" s="9" t="n">
-        <v>68020787</v>
+        <v>319983894</v>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -7221,13 +7211,13 @@
         <v>3</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>423288615</v>
+        <v>392285593</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>146817603</v>
+        <v>115814581</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7536,34 +7526,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>872</v>
+        <v>853</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>103492155254</v>
+        <v>101567060620</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>519</v>
+        <v>500</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>65672621999</v>
+        <v>63747527365</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>519</v>
+        <v>500</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>64069051567.41</v>
+        <v>62774573010.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>308</v>
+        <v>290</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>37942026823.02</v>
+        <v>36832148266.02</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>1028156578</v>
+        <v>680948578</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>353</v>
@@ -8371,28 +8361,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F17" s="11" t="n">
-        <v>26735477939</v>
+        <v>25286544212</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H17" s="11" t="n">
-        <v>26394591741</v>
+        <v>24598091741</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J17" s="11" t="n">
-        <v>26394591741</v>
+        <v>24598091741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8478,29 +8468,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="11" t="n">
-        <v>201600000</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="11" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="11" t="n">
-        <v>199078500</v>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -8532,29 +8538,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>1090890000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>1081900000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>1081900000</v>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -8590,13 +8612,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>1269914370</v>
+        <v>634957185</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8644,7 +8666,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
@@ -8690,7 +8712,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>277500000</v>
+        <v>272000000</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -8823,34 +8845,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>48003814160</v>
+        <v>5652342335</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>47632716881</v>
+        <v>5281245056</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>4157004750</v>
+        <v>2971571974</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>2945468782</v>
+        <v>1854621974</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -9507,34 +9529,38 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>5934990898</v>
+        <v>5061390898</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>2946694000</v>
+        <v>2073094000</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>2509890630</v>
+        <v>2073094000</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>2509890630</v>
-      </c>
-      <c r="K37" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" s="11" t="n">
-        <v>436796630</v>
+        <v>2073094000</v>
+      </c>
+      <c r="K37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M37" s="4" t="n">
         <v>4</v>
@@ -9850,13 +9876,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>346000000</v>
+        <v>328338000</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -11777,28 +11803,28 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D72" s="9" t="n">
-        <v>14398798637</v>
+        <v>7792798637</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>8054692000</v>
+        <v>1448692000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>2808340212</v>
+        <v>607099212</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>2</v>
@@ -12041,40 +12067,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>240</v>
+        <v>210</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>184489493359</v>
+        <v>131258878622</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>161</v>
+        <v>131</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>145779681118</v>
+        <v>92554566381</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>161</v>
+        <v>131</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>70786680805.01001</v>
+        <v>63885731899.01</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>66338247005</v>
+        <v>59437298099</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>4005987066</v>
+        <v>2478343628</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>79</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>38709812241</v>
+        <v>38704312241</v>
       </c>
     </row>
   </sheetData>
@@ -13063,13 +13089,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>5040000000</v>
+        <v>4988300000</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
@@ -13113,29 +13139,45 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="9" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="E20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="9" t="n">
-        <v>2688000000</v>
-      </c>
-      <c r="G20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>2646500000</v>
-      </c>
-      <c r="I20" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>2646500000</v>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -13518,28 +13560,40 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D26" s="9" t="n">
-        <v>5399320575</v>
-      </c>
-      <c r="E26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="F26" s="9" t="n">
-        <v>2700000000</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="9" t="n">
-        <v>2699298000</v>
-      </c>
-      <c r="I26" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="9" t="n">
-        <v>2699298000</v>
+        <v>2699320575</v>
+      </c>
+      <c r="E26" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I26" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K26" s="10" t="inlineStr">
         <is>
@@ -16982,28 +17036,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>278721235553</v>
+        <v>273281535553</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>147115370800</v>
+        <v>141675670800</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>65889582008.97</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>71235380008.97</v>
+        <v>65889582008.97</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Auto update Pengadaan 2026-10-15 10:09:56
</commit_message>
<xml_diff>
--- a/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-15).xlsx
+++ b/output/tepra/2026/Tepra Kobar_Progres PBJ tahun 2026 (2026-10-15).xlsx
@@ -1020,27 +1020,35 @@
           <t>DINAS PEKERJAAN UMUM DAN PENATAAN RUANG - 1.03.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C17" s="4" t="n">
-        <v>1</v>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E17" s="4" t="n">
-        <v>1</v>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G17" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>1796500000</v>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
@@ -1162,27 +1170,35 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="7" t="n">
-        <v>3</v>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="E20" s="7" t="n">
-        <v>3</v>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F20" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G20" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" s="9" t="n">
-        <v>3839600910</v>
+      <c r="G20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I20" s="10" t="inlineStr">
         <is>
@@ -1308,13 +1324,13 @@
         <v>80</v>
       </c>
       <c r="D23" s="11" t="n">
-        <v>850708644</v>
+        <v>847942644</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F23" s="11" t="n">
-        <v>62227794</v>
+        <v>59461794</v>
       </c>
       <c r="G23" s="4" t="n">
         <v>5</v>
@@ -1373,22 +1389,22 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>128</v>
+        <v>103</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>674360508</v>
+        <v>677290237</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>134654115</v>
+        <v>137583844</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>1345382085</v>
+        <v>116218702</v>
       </c>
       <c r="I25" s="4" t="n">
         <v>90</v>
@@ -1407,22 +1423,22 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D26" s="9" t="n">
         <v>507942073</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F26" s="9" t="n">
         <v>338217900</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H26" s="9" t="n">
-        <v>3037348900</v>
+        <v>338050900</v>
       </c>
       <c r="I26" s="7" t="n">
         <v>22</v>
@@ -1444,13 +1460,13 @@
         <v>130</v>
       </c>
       <c r="D27" s="11" t="n">
-        <v>990746345</v>
+        <v>993618445</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>41</v>
       </c>
       <c r="F27" s="11" t="n">
-        <v>348242988</v>
+        <v>351115088</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>41</v>
@@ -1512,13 +1528,13 @@
         <v>171</v>
       </c>
       <c r="D29" s="11" t="n">
-        <v>2260066920</v>
+        <v>2269571073</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>54</v>
       </c>
       <c r="F29" s="11" t="n">
-        <v>1126736515</v>
+        <v>1136240668</v>
       </c>
       <c r="G29" s="4" t="n">
         <v>54</v>
@@ -1543,22 +1559,22 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" s="9" t="n">
         <v>367878502</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F30" s="9" t="n">
         <v>79101092</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>225945607</v>
+        <v>75945607</v>
       </c>
       <c r="I30" s="7" t="n">
         <v>49</v>
@@ -1580,13 +1596,13 @@
         <v>55</v>
       </c>
       <c r="D31" s="11" t="n">
-        <v>335468518</v>
+        <v>335612543</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F31" s="11" t="n">
-        <v>30118025</v>
+        <v>30262050</v>
       </c>
       <c r="G31" s="4" t="n">
         <v>5</v>
@@ -1614,13 +1630,13 @@
         <v>122</v>
       </c>
       <c r="D32" s="9" t="n">
-        <v>764274671</v>
+        <v>767894130</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>6</v>
       </c>
       <c r="F32" s="9" t="n">
-        <v>103722907</v>
+        <v>107342366</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>6</v>
@@ -1648,13 +1664,13 @@
         <v>42</v>
       </c>
       <c r="D33" s="11" t="n">
-        <v>204513748</v>
+        <v>292846882</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>5</v>
       </c>
       <c r="F33" s="11" t="n">
-        <v>20641550</v>
+        <v>108974684</v>
       </c>
       <c r="G33" s="4" t="n">
         <v>5</v>
@@ -1716,13 +1732,13 @@
         <v>66</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>463836830</v>
+        <v>463972148</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>6</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>93231105</v>
+        <v>93366423</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>6</v>
@@ -1781,22 +1797,22 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>111</v>
+        <v>100</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>847360391</v>
+        <v>1227952291</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>81094602</v>
+        <v>461686502</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1801299990</v>
+        <v>451166160</v>
       </c>
       <c r="I37" s="4" t="n">
         <v>84</v>
@@ -1818,13 +1834,13 @@
         <v>97</v>
       </c>
       <c r="D38" s="9" t="n">
-        <v>382731831</v>
+        <v>384332451</v>
       </c>
       <c r="E38" s="7" t="n">
         <v>11</v>
       </c>
       <c r="F38" s="9" t="n">
-        <v>85740718</v>
+        <v>87341338</v>
       </c>
       <c r="G38" s="7" t="n">
         <v>11</v>
@@ -1852,13 +1868,13 @@
         <v>107</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>1245457621</v>
+        <v>1270987621</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>18</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>352528156</v>
+        <v>378058156</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>18</v>
@@ -1920,13 +1936,13 @@
         <v>82</v>
       </c>
       <c r="D41" s="11" t="n">
-        <v>724469682</v>
+        <v>737837746</v>
       </c>
       <c r="E41" s="4" t="n">
         <v>16</v>
       </c>
       <c r="F41" s="11" t="n">
-        <v>59693782</v>
+        <v>73061846</v>
       </c>
       <c r="G41" s="4" t="n">
         <v>16</v>
@@ -1988,13 +2004,13 @@
         <v>50</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>727698127</v>
+        <v>708077545</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>54570486</v>
+        <v>34949904</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>3</v>
@@ -2019,22 +2035,22 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D44" s="9" t="n">
         <v>282819298</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F44" s="9" t="n">
         <v>151137140</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>83626512</v>
+        <v>72726534</v>
       </c>
       <c r="I44" s="7" t="n">
         <v>15</v>
@@ -2103,22 +2119,22 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>1174814171</v>
+        <v>1126161761</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F46" s="9" t="n">
-        <v>173625311</v>
+        <v>124972901</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="H46" s="9" t="n">
-        <v>318350703</v>
+        <v>121983128</v>
       </c>
       <c r="I46" s="7" t="n">
         <v>169</v>
@@ -2224,13 +2240,13 @@
         <v>105</v>
       </c>
       <c r="D49" s="11" t="n">
-        <v>618221476</v>
+        <v>620146476</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>15</v>
       </c>
       <c r="F49" s="11" t="n">
-        <v>203015123</v>
+        <v>204940123</v>
       </c>
       <c r="G49" s="4" t="n">
         <v>15</v>
@@ -2339,24 +2355,30 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D52" s="9" t="n">
         <v>111669795</v>
       </c>
-      <c r="E52" s="7" t="n">
-        <v>3</v>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="F52" s="10" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G52" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H52" s="9" t="n">
-        <v>68020787</v>
+      <c r="G52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H52" s="10" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="I52" s="7" t="n">
         <v>14</v>
@@ -2882,13 +2904,13 @@
         <v>32</v>
       </c>
       <c r="D65" s="11" t="n">
-        <v>199016800</v>
+        <v>197795800</v>
       </c>
       <c r="E65" s="4" t="n">
         <v>8</v>
       </c>
       <c r="F65" s="11" t="n">
-        <v>47156987</v>
+        <v>45935987</v>
       </c>
       <c r="G65" s="4" t="n">
         <v>8</v>
@@ -3126,13 +3148,13 @@
         <v>20</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>174734876</v>
+        <v>181625201</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>28826575</v>
+        <v>35716900</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>2</v>
@@ -3157,22 +3179,22 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D72" s="9" t="n">
         <v>637283463</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F72" s="9" t="n">
         <v>108000000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>2359971000</v>
+        <v>158730000</v>
       </c>
       <c r="I72" s="7" t="n">
         <v>29</v>
@@ -3278,7 +3300,7 @@
         <v>92</v>
       </c>
       <c r="D75" s="11" t="n">
-        <v>1054602496</v>
+        <v>1089002496</v>
       </c>
       <c r="E75" s="4" t="n">
         <v>18</v>
@@ -3296,7 +3318,7 @@
         <v>74</v>
       </c>
       <c r="J75" s="11" t="n">
-        <v>634728310</v>
+        <v>669128310</v>
       </c>
     </row>
     <row r="76" ht="45" customHeight="1">
@@ -3312,13 +3334,13 @@
         <v>151</v>
       </c>
       <c r="D76" s="9" t="n">
-        <v>1480218770</v>
+        <v>1482468770</v>
       </c>
       <c r="E76" s="7" t="n">
         <v>26</v>
       </c>
       <c r="F76" s="9" t="n">
-        <v>213985114</v>
+        <v>216235114</v>
       </c>
       <c r="G76" s="7" t="n">
         <v>26</v>
@@ -3341,28 +3363,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>3955</v>
+        <v>3904</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>32283625052</v>
+        <v>32785458887</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>477</v>
+        <v>426</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>6329164221</v>
+        <v>6796598056</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>477</v>
+        <v>426</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>19914588683.6</v>
+        <v>6373363220.6</v>
       </c>
       <c r="I77" s="12" t="n">
         <v>3478</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>25954460831</v>
+        <v>25988860831</v>
       </c>
     </row>
   </sheetData>
@@ -3783,13 +3805,13 @@
         <v>5</v>
       </c>
       <c r="D11" s="11" t="n">
-        <v>413165330</v>
+        <v>428765330</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="11" t="n">
-        <v>261110330</v>
+        <v>276710330</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>3</v>
@@ -4223,29 +4245,45 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D19" s="11" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="E19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="11" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="G19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="11" t="n">
-        <v>199078500</v>
-      </c>
-      <c r="I19" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="11" t="n">
-        <v>199078500</v>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -4277,45 +4315,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>112000000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>112000000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>111200910</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>111200910</v>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -4584,28 +4606,28 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>1346095756</v>
+        <v>1566751699</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>1004886595</v>
+        <v>1225542538</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>852531955</v>
+        <v>896262562</v>
       </c>
       <c r="K25" s="4" t="n">
         <v>4</v>
@@ -4830,28 +4852,28 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D30" s="9" t="n">
-        <v>388286000</v>
+        <v>538286000</v>
       </c>
       <c r="E30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="9" t="n">
-        <v>138750000</v>
+        <v>288750000</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="I30" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J30" s="9" t="n">
-        <v>138306000</v>
+        <v>288306000</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
@@ -5083,13 +5105,13 @@
         <v>13</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>1667542131</v>
+        <v>1694840343</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F35" s="11" t="n">
-        <v>885723156</v>
+        <v>913021368</v>
       </c>
       <c r="G35" s="4" t="n">
         <v>7</v>
@@ -5180,34 +5202,34 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>2613177050</v>
+        <v>3541045550</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>1097221951</v>
+        <v>2025090451</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>1062482323</v>
+        <v>1975819523</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>852976373</v>
+        <v>1581713573</v>
       </c>
       <c r="K37" s="4" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L37" s="11" t="n">
-        <v>188207363</v>
+        <v>535415363</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>16</v>
@@ -5291,13 +5313,13 @@
         <v>37</v>
       </c>
       <c r="D39" s="11" t="n">
-        <v>4277601639</v>
+        <v>4288626639</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>24</v>
       </c>
       <c r="F39" s="11" t="n">
-        <v>2758359586</v>
+        <v>2769384586</v>
       </c>
       <c r="G39" s="4" t="n">
         <v>24</v>
@@ -5562,28 +5584,28 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D44" s="9" t="n">
-        <v>523391100</v>
+        <v>595373450</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F44" s="9" t="n">
-        <v>345935300</v>
+        <v>417917650</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="I44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>187868022</v>
+        <v>198768000</v>
       </c>
       <c r="K44" s="10" t="inlineStr">
         <is>
@@ -5682,28 +5704,28 @@
         </is>
       </c>
       <c r="C46" s="7" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D46" s="9" t="n">
-        <v>716222170</v>
+        <v>932380105</v>
       </c>
       <c r="E46" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F46" s="9" t="n">
+        <v>471330601</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H46" s="9" t="n">
+        <v>448555830</v>
+      </c>
+      <c r="I46" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="F46" s="9" t="n">
-        <v>255172666</v>
-      </c>
-      <c r="G46" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="H46" s="9" t="n">
-        <v>252188255</v>
-      </c>
-      <c r="I46" s="7" t="n">
-        <v>2</v>
-      </c>
       <c r="J46" s="9" t="n">
-        <v>113248255</v>
+        <v>309615830</v>
       </c>
       <c r="K46" s="10" t="inlineStr">
         <is>
@@ -6026,40 +6048,28 @@
         </is>
       </c>
       <c r="C52" s="7" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D52" s="9" t="n">
-        <v>319983894</v>
-      </c>
-      <c r="E52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J52" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>660566066</v>
+      </c>
+      <c r="E52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" s="9" t="n">
+        <v>340582172</v>
+      </c>
+      <c r="G52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H52" s="9" t="n">
+        <v>68020787</v>
+      </c>
+      <c r="I52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="9" t="n">
+        <v>68020787</v>
       </c>
       <c r="K52" s="10" t="inlineStr">
         <is>
@@ -7211,13 +7221,13 @@
         <v>3</v>
       </c>
       <c r="D71" s="11" t="n">
-        <v>392285593</v>
+        <v>423288615</v>
       </c>
       <c r="E71" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F71" s="11" t="n">
-        <v>115814581</v>
+        <v>146817603</v>
       </c>
       <c r="G71" s="4" t="n">
         <v>1</v>
@@ -7526,34 +7536,34 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>853</v>
+        <v>872</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>101567060620</v>
+        <v>103492155254</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>500</v>
+        <v>519</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>63747527365</v>
+        <v>65672621999</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>500</v>
+        <v>519</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>62774573010.41</v>
+        <v>64069051567.41</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>290</v>
+        <v>308</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>36832148266.02</v>
+        <v>37942026823.02</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>680948578</v>
+        <v>1028156578</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>353</v>
@@ -8361,28 +8371,28 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="E17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>26735477939</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="H17" s="11" t="n">
+        <v>26394591741</v>
+      </c>
+      <c r="I17" s="4" t="n">
         <v>22</v>
       </c>
-      <c r="D17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="E17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="F17" s="11" t="n">
-        <v>25286544212</v>
-      </c>
-      <c r="G17" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="H17" s="11" t="n">
-        <v>24598091741</v>
-      </c>
-      <c r="I17" s="4" t="n">
-        <v>21</v>
-      </c>
       <c r="J17" s="11" t="n">
-        <v>24598091741</v>
+        <v>26394591741</v>
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
@@ -8468,45 +8478,29 @@
           <t>DINAS PERHUBUNGAN - 2.15.0.00.0.00.01.0000</t>
         </is>
       </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="11" t="n">
+        <v>201600000</v>
+      </c>
+      <c r="E19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="11" t="n">
+        <v>201600000</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="11" t="n">
+        <v>199078500</v>
+      </c>
+      <c r="I19" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="11" t="n">
+        <v>199078500</v>
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
@@ -8538,45 +8532,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>1090890000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>1090890000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>1081900000</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>1081900000</v>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -8612,13 +8590,13 @@
         <v>1</v>
       </c>
       <c r="D21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="11" t="n">
-        <v>634957185</v>
+        <v>1269914370</v>
       </c>
       <c r="G21" s="4" t="n">
         <v>1</v>
@@ -8666,7 +8644,7 @@
         <v>1</v>
       </c>
       <c r="D22" s="9" t="n">
-        <v>272000000</v>
+        <v>277500000</v>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
@@ -8712,7 +8690,7 @@
         <v>1</v>
       </c>
       <c r="N22" s="9" t="n">
-        <v>272000000</v>
+        <v>277500000</v>
       </c>
     </row>
     <row r="23" ht="45" customHeight="1">
@@ -8845,34 +8823,34 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D25" s="11" t="n">
-        <v>5652342335</v>
+        <v>48003814160</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="F25" s="11" t="n">
-        <v>5281245056</v>
+        <v>47632716881</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="H25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>9</v>
+        <v>32</v>
       </c>
       <c r="J25" s="11" t="n">
-        <v>2971571974</v>
+        <v>4157004750</v>
       </c>
       <c r="K25" s="4" t="n">
-        <v>6</v>
+        <v>27</v>
       </c>
       <c r="L25" s="11" t="n">
-        <v>1854621974</v>
+        <v>2945468782</v>
       </c>
       <c r="M25" s="4" t="n">
         <v>1</v>
@@ -9529,38 +9507,34 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D37" s="11" t="n">
-        <v>5061390898</v>
+        <v>5934990898</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F37" s="11" t="n">
-        <v>2073094000</v>
+        <v>2946694000</v>
       </c>
       <c r="G37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H37" s="11" t="n">
-        <v>2073094000</v>
+        <v>2509890630</v>
       </c>
       <c r="I37" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J37" s="11" t="n">
-        <v>2073094000</v>
-      </c>
-      <c r="K37" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L37" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>2509890630</v>
+      </c>
+      <c r="K37" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L37" s="11" t="n">
+        <v>436796630</v>
       </c>
       <c r="M37" s="4" t="n">
         <v>4</v>
@@ -9876,13 +9850,13 @@
         <v>1</v>
       </c>
       <c r="D43" s="11" t="n">
-        <v>328338000</v>
+        <v>346000000</v>
       </c>
       <c r="E43" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F43" s="11" t="n">
-        <v>328338000</v>
+        <v>346000000</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>1</v>
@@ -11803,28 +11777,28 @@
         </is>
       </c>
       <c r="C72" s="7" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D72" s="9" t="n">
-        <v>7792798637</v>
+        <v>14398798637</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F72" s="9" t="n">
-        <v>1448692000</v>
+        <v>8054692000</v>
       </c>
       <c r="G72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H72" s="9" t="n">
-        <v>607099212</v>
+        <v>2808340212</v>
       </c>
       <c r="I72" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="J72" s="9" t="n">
-        <v>607099212</v>
+        <v>2808340212</v>
       </c>
       <c r="K72" s="7" t="n">
         <v>2</v>
@@ -12067,40 +12041,40 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>210</v>
+        <v>240</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>131258878622</v>
+        <v>184489493359</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>92554566381</v>
+        <v>145779681118</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>131</v>
+        <v>161</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>63885731899.01</v>
+        <v>70786680805.01001</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>59437298099</v>
+        <v>66338247005</v>
       </c>
       <c r="K77" s="12" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="L77" s="13" t="n">
-        <v>2478343628</v>
+        <v>4005987066</v>
       </c>
       <c r="M77" s="12" t="n">
         <v>79</v>
       </c>
       <c r="N77" s="13" t="n">
-        <v>38704312241</v>
+        <v>38709812241</v>
       </c>
     </row>
   </sheetData>
@@ -13089,13 +13063,13 @@
         <v>1</v>
       </c>
       <c r="D19" s="11" t="n">
-        <v>4988300000</v>
+        <v>5040000000</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="11" t="n">
-        <v>4988300000</v>
+        <v>5040000000</v>
       </c>
       <c r="G19" s="4" t="n">
         <v>1</v>
@@ -13139,45 +13113,29 @@
           <t>DINAS PERINDUSTRIAN, PERDAGANGAN, KOPERASI, USAHA KECIL DAN MENENGAH - 2.17.3.30.3.31.01.0000</t>
         </is>
       </c>
-      <c r="C20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J20" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="C20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="9" t="n">
+        <v>2688000000</v>
+      </c>
+      <c r="E20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>2688000000</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="9" t="n">
+        <v>2646500000</v>
+      </c>
+      <c r="I20" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>2646500000</v>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
@@ -13560,40 +13518,28 @@
         </is>
       </c>
       <c r="C26" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="9" t="n">
+        <v>5399320575</v>
+      </c>
+      <c r="E26" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="D26" s="9" t="n">
-        <v>2699320575</v>
-      </c>
-      <c r="E26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" s="10" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="F26" s="9" t="n">
+        <v>2700000000</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="9" t="n">
+        <v>2699298000</v>
+      </c>
+      <c r="I26" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>2699298000</v>
       </c>
       <c r="K26" s="10" t="inlineStr">
         <is>
@@ -17036,28 +16982,28 @@
         </is>
       </c>
       <c r="C77" s="12" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D77" s="13" t="n">
-        <v>273281535553</v>
+        <v>278721235553</v>
       </c>
       <c r="E77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F77" s="13" t="n">
-        <v>141675670800</v>
+        <v>147115370800</v>
       </c>
       <c r="G77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>65889582008.97</v>
+        <v>71235380008.97</v>
       </c>
       <c r="I77" s="12" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J77" s="13" t="n">
-        <v>65889582008.97</v>
+        <v>71235380008.97</v>
       </c>
       <c r="K77" s="2" t="inlineStr">
         <is>

</xml_diff>